<commit_message>
Avance en el analisis de los datos del primer trimestre del 2026
</commit_message>
<xml_diff>
--- a/data/raw/q1_2026/Ingresos - 1er Quarter 2026.xlsx
+++ b/data/raw/q1_2026/Ingresos - 1er Quarter 2026.xlsx
@@ -79,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -105,7 +105,13 @@
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -546,23 +552,23 @@
       <c r="B12" s="2">
         <v>46111.0</v>
       </c>
-      <c r="C12" s="3">
-        <v>74000.0</v>
+      <c r="C12" s="8">
+        <v>71000.0</v>
       </c>
       <c r="D12" s="3">
         <v>90100.0</v>
       </c>
       <c r="E12" s="6">
         <f t="shared" si="2"/>
-        <v>-0.1786903441</v>
+        <v>-0.2119866815</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="8"/>
+      <c r="C13" s="9"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="6"/>
+      <c r="E13" s="10"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>